<commit_message>
更新日报: 2026/09/07 周一 17:25:25.08
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FC725A-2F14-49DE-B4F8-5E6826124926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE10896C-4253-4AA7-894F-8475DA1A5A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -460,32 +460,28 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>2026年8月31日-2026年9月4日</t>
+    <t>2026年9月7日-2026年9月11日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等
-2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写
+1. 学习了数据集成的进阶操作 学习了增量迁移的原理介绍 以及四种增量迁移方式: 文件 关系数据库 HBase/CloudTable和MongoDB/DDS增量迁移
+2. 学习了时间宏变量使用解析
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-学习数据集成CDM如何离线作业
+学习如何优化迁移性能章节
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月4日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>周一:
-1. 学习了GDC的基本功能 对GDC有了初步的了解 
-2. 学习GDC数据迁移的产品文档中迁移相关的章节 并且仔细学习了一个GDC数据迁移的使用案例
+1. 学习了数据集成的进阶操作 学习了增量迁移的原理介绍 以及四种增量迁移方式: 文件 关系数据库 HBase/CloudTable和MongoDB/DDS增量迁移
+2. 学习了时间宏变量使用解析
 周二:
 1. 在大唐机房做了验收指南中的租户与VDC中的创建租户 VDC 创建VDC管理员等等 还有运维管理中的资源回收站 告警处理 运维监控等测试
 周三:
@@ -495,6 +491,10 @@
 周五:
 1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等 使用OBS桶或者将作业 配置和脚本等压缩成zip文件导出到本地 然后在新的工作空间导入
 2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>工作&amp;学习日报-9月7日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1228,6 +1228,93 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1281,97 +1368,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2122,7 +2122,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2227,154 +2227,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="47"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="47"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="58"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
+      <c r="A6" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2383,17 +2383,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="43"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="34"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2411,15 +2411,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2429,82 +2429,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="28"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="35"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="22"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2514,6 +2497,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/08 周二 17:24:48.10
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE10896C-4253-4AA7-894F-8475DA1A5A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A36BA4D-87C8-4FEA-8A87-C28D84A2704E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.日工作简报" sheetId="11" r:id="rId1"/>
@@ -464,16 +464,20 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>工作&amp;学习日报-9月8日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>重点工作: 
-1. 学习了数据集成的进阶操作 学习了增量迁移的原理介绍 以及四种增量迁移方式: 文件 关系数据库 HBase/CloudTable和MongoDB/DDS增量迁移
-2. 学习了时间宏变量使用解析
+进行dgc验收测试指南里内容的测试
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-学习如何优化迁移性能章节
+1. 学习了DataArts Studio的实例发放和工作空间资源划分的实践操作 包含了如何表行数和库大小 通过数据质量对比迁移前后的结果
+以及如何处理数据开发中的告警
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -483,7 +487,7 @@
 1. 学习了数据集成的进阶操作 学习了增量迁移的原理介绍 以及四种增量迁移方式: 文件 关系数据库 HBase/CloudTable和MongoDB/DDS增量迁移
 2. 学习了时间宏变量使用解析
 周二:
-1. 在大唐机房做了验收指南中的租户与VDC中的创建租户 VDC 创建VDC管理员等等 还有运维管理中的资源回收站 告警处理 运维监控等测试
+1. 学习了DataArts Studio的实例发放和工作空间资源划分的实践操作 包含了如何表行数和库大小 通过数据质量对比迁移前后的结果以及如何处理数据开发中的告警
 周三:
 1. 继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试
 周四:
@@ -491,10 +495,6 @@
 周五:
 1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等 使用OBS桶或者将作业 配置和脚本等压缩成zip文件导出到本地 然后在新的工作空间导入
 2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>工作&amp;学习日报-9月7日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1228,37 +1228,141 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1285,130 +1389,26 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2121,74 +2121,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
+      <c r="A1" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="68" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="70"/>
+      <c r="A3" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="23"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="71" t="s">
+      <c r="A5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="72"/>
-      <c r="D5" s="72"/>
-      <c r="E5" s="72"/>
-      <c r="F5" s="72"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="73"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="62"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="64"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2227,154 +2227,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="69"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="59"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="70"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="73"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="59"/>
+      <c r="H4" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="62"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="65"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="A6" s="66" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="52"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="53"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="50"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="53"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="50"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2383,17 +2383,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="55"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="46"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2411,15 +2411,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="36"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="37"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2429,65 +2429,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="40"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="42"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="47"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="32"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2497,23 +2514,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/09 周三 17:46:01.02
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A36BA4D-87C8-4FEA-8A87-C28D84A2704E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8B4B2E-BE42-4C79-99D4-C3C6174DA45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,20 +464,20 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月8日</t>
+    <t>工作&amp;学习日报-9月9日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-进行dgc验收测试指南里内容的测试
+1. 做了数据治理中心的验收测试文档 我主要干的是数据开发的测试 包括dws hive spark和主机连接的创建 还有配置管理 包括新建jar file archive 环境变量登资源
+2. 还有脚本开发 包括dws flink python spark hive shell脚本的测试 脚本目录的重命名 移动 删除等操作
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 学习了DataArts Studio的实例发放和工作空间资源划分的实践操作 包含了如何表行数和库大小 通过数据质量对比迁移前后的结果
-以及如何处理数据开发中的告警
+进行数据治理验收测试
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -489,7 +489,8 @@
 周二:
 1. 学习了DataArts Studio的实例发放和工作空间资源划分的实践操作 包含了如何表行数和库大小 通过数据质量对比迁移前后的结果以及如何处理数据开发中的告警
 周三:
-1. 继续做了验收测试指南 包括单点CCAE FusionCare日常巡检 创建主门户 创建策略 以及弹性云服务器申请 注册镜像 以及各种云硬盘操作 以及对象存储服务的测试
+1. 1. 做了数据治理中心的验收测试文档 我主要干的是数据开发的测试 包括dws hive spark和主机连接的创建 还有配置管理 包括新建jar file archive 环境变量登资源
+2. 还有脚本开发 包括dws flink python spark hive shell脚本的测试 脚本目录的重命名 移动 删除等操作
 周四:
 1. 学习数据迁移过程 首先迁移DGC的脚本 配置和作业等内容然后使用DGC这个迁移工具 批量迁移MRS和DWS的数据
 周五:
@@ -1228,6 +1229,152 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1263,152 +1410,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="166">
@@ -2121,74 +2122,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
-      <c r="A3" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="23"/>
+      <c r="A3" s="68" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="70"/>
     </row>
     <row r="4" spans="1:8" ht="54.75" customHeight="1">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26"/>
+      <c r="A5" s="71" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="73"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2227,154 +2228,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="69"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="59"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="58" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="59"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="59" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="59"/>
-      <c r="J2" s="70"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="57" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="71" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="72"/>
-      <c r="J3" s="73"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="58" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="59"/>
-      <c r="H4" s="60" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="61"/>
-      <c r="J4" s="62"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="65"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="53"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="50"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="53"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="50"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2383,17 +2384,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="55"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="46"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2411,15 +2412,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="36"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="37"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2429,82 +2430,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="40"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="45"/>
-      <c r="G13" s="46"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="44" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="47"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="30" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="32"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="33" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="34"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2514,6 +2498,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/10 周四 17:44:59.06
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8B4B2E-BE42-4C79-99D4-C3C6174DA45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED9FAE7-DEAB-4CF7-BFAB-F1C54DA9986B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,20 +464,20 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月9日</t>
+    <t>工作&amp;学习日报-9月10日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 做了数据治理中心的验收测试文档 我主要干的是数据开发的测试 包括dws hive spark和主机连接的创建 还有配置管理 包括新建jar file archive 环境变量登资源
-2. 还有脚本开发 包括dws flink python spark hive shell脚本的测试 脚本目录的重命名 移动 删除等操作
+1. 进行数据治理的验收测试 主要做的是数据架构验收用例: 比如添加审核人 创建流程设计 导入 导出 删除 创建主题设计 还有概念模型的创建
+2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-进行数据治理验收测试
+进行源端和CDM的网络连通测试
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -492,7 +492,8 @@
 1. 1. 做了数据治理中心的验收测试文档 我主要干的是数据开发的测试 包括dws hive spark和主机连接的创建 还有配置管理 包括新建jar file archive 环境变量登资源
 2. 还有脚本开发 包括dws flink python spark hive shell脚本的测试 脚本目录的重命名 移动 删除等操作
 周四:
-1. 学习数据迁移过程 首先迁移DGC的脚本 配置和作业等内容然后使用DGC这个迁移工具 批量迁移MRS和DWS的数据
+1. 1. 进行数据治理的验收测试 主要做的是数据架构验收用例: 比如添加审核人 创建流程设计 导入 导出 删除 创建主题设计 还有概念模型的创建
+2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
 周五:
 1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等 使用OBS桶或者将作业 配置和脚本等压缩成zip文件导出到本地 然后在新的工作空间导入
 2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写</t>
@@ -1229,37 +1230,105 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1286,93 +1355,25 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2228,154 +2229,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2384,17 +2385,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2412,15 +2413,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2430,65 +2431,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2498,23 +2516,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/11 周五 19:03:14.36
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED9FAE7-DEAB-4CF7-BFAB-F1C54DA9986B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B29703-1045-4770-AA25-C17BE4118F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,20 +464,19 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月10日</t>
+    <t>工作&amp;学习日报-9月11日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 进行数据治理的验收测试 主要做的是数据架构验收用例: 比如添加审核人 创建流程设计 导入 导出 删除 创建主题设计 还有概念模型的创建
-2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
+1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-进行源端和CDM的网络连通测试
+1. 继续进行数据服务里的dt_sub_nmnt_prd这个工作空间的API的发布和授权操作 
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -495,8 +494,7 @@
 1. 1. 进行数据治理的验收测试 主要做的是数据架构验收用例: 比如添加审核人 创建流程设计 导入 导出 删除 创建主题设计 还有概念模型的创建
 2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
 周五:
-1. 学习了DataArts Studio资源迁移的全过程 以及约束条件 迁移选择的工具等 使用OBS桶或者将作业 配置和脚本等压缩成zip文件导出到本地 然后在新的工作空间导入
-2. 学习DataArts Studio支持的数据源包括哪些 以及连接参数怎么写</t>
+1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1230,6 +1228,93 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1283,97 +1368,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2229,154 +2227,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="47"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="47"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="58"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2385,17 +2383,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="43"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="34"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2413,15 +2411,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2431,82 +2429,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="28"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="35"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="22"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2516,6 +2497,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/14 周一 17:56:53.36
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B29703-1045-4770-AA25-C17BE4118F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBFBA145-E02F-4F47-9123-D25DEC80C299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -460,31 +460,28 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>2026年9月7日-2026年9月11日</t>
+    <t>工作&amp;学习日报-9月14日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月11日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>重点工作: 
-1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试
+1. 进行了源端和CDM集群的网络连通行测试
+2. 进行了数据库到源端的连通性 并做了连接 包括oracle postgresql和DM数据库的连接
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 继续进行数据服务里的dt_sub_nmnt_prd这个工作空间的API的发布和授权操作 
+1. 学习DGC作业迁移的流程
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>周一:
-1. 学习了数据集成的进阶操作 学习了增量迁移的原理介绍 以及四种增量迁移方式: 文件 关系数据库 HBase/CloudTable和MongoDB/DDS增量迁移
-2. 学习了时间宏变量使用解析
+1. 进行了源端和CDM集群的网络连通行测试
+2. 进行了数据库到源端的连通性 并做了连接 包括oracle postgresql和DM数据库的连接
 周二:
 1. 学习了DataArts Studio的实例发放和工作空间资源划分的实践操作 包含了如何表行数和库大小 通过数据质量对比迁移前后的结果以及如何处理数据开发中的告警
 周三:
@@ -495,6 +492,10 @@
 2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
 周五:
 1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026年9月14日-2026年9月18日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1228,37 +1229,105 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1285,93 +1354,25 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2122,7 +2123,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2146,7 +2147,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2170,7 +2171,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2227,154 +2228,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="H2" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="A6" s="54" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2383,17 +2384,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2411,15 +2412,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2429,65 +2430,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2497,23 +2515,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/15 周二 18:00:08.60
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBFBA145-E02F-4F47-9123-D25DEC80C299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA630952-545E-490A-A555-D63A5FCC7E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -460,20 +460,24 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月14日</t>
+    <t>2026年9月14日-2026年9月18日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>工作&amp;学习日报-9月15日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>重点工作: 
-1. 进行了源端和CDM集群的网络连通行测试
-2. 进行了数据库到源端的连通性 并做了连接 包括oracle postgresql和DM数据库的连接
+1. 进行了源端到cdm集群端的网络和端口测试
+2. 从运营面进入数据治理中心  选择工作空间 然后进入数据集成 把dgc里的作业导入到cdm中
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 学习DGC作业迁移的流程
+1. 继续进行dgc迁移工作
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -483,7 +487,8 @@
 1. 进行了源端和CDM集群的网络连通行测试
 2. 进行了数据库到源端的连通性 并做了连接 包括oracle postgresql和DM数据库的连接
 周二:
-1. 学习了DataArts Studio的实例发放和工作空间资源划分的实践操作 包含了如何表行数和库大小 通过数据质量对比迁移前后的结果以及如何处理数据开发中的告警
+1. 进行了源端到cdm集群端的网络和端口测试
+2. 从运营面进入数据治理中心  选择工作空间 然后进入数据集成 把dgc里的作业导入到cdm中
 周三:
 1. 1. 做了数据治理中心的验收测试文档 我主要干的是数据开发的测试 包括dws hive spark和主机连接的创建 还有配置管理 包括新建jar file archive 环境变量登资源
 2. 还有脚本开发 包括dws flink python spark hive shell脚本的测试 脚本目录的重命名 移动 删除等操作
@@ -492,10 +497,6 @@
 2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
 周五:
 1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026年9月14日-2026年9月18日</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1229,6 +1230,93 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1282,97 +1370,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2123,7 +2124,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2147,7 +2148,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2171,7 +2172,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2228,154 +2229,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="47"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="47"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="47" t="s">
-        <v>40</v>
-      </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="58"/>
+      <c r="H2" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="54" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
+      <c r="A6" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2384,17 +2385,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="43"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="34"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2412,15 +2413,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2430,82 +2431,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="28"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="35"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="22"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2515,6 +2499,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/16 周三 17:25:53.24
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA630952-545E-490A-A555-D63A5FCC7E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B4155A-E223-4220-BB6B-DEDF83FCB6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,20 +464,20 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月15日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>重点工作: 
-1. 进行了源端到cdm集群端的网络和端口测试
-2. 从运营面进入数据治理中心  选择工作空间 然后进入数据集成 把dgc里的作业导入到cdm中
+1. 继续进行dgc迁移工作
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>工作&amp;学习日报-9月16日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>重点工作: 
-1. 继续进行dgc迁移工作
+1. 继续对不通的网络进行重新测试
+2. 学习dgc迁移的其他理论知识
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -490,8 +490,8 @@
 1. 进行了源端到cdm集群端的网络和端口测试
 2. 从运营面进入数据治理中心  选择工作空间 然后进入数据集成 把dgc里的作业导入到cdm中
 周三:
-1. 1. 做了数据治理中心的验收测试文档 我主要干的是数据开发的测试 包括dws hive spark和主机连接的创建 还有配置管理 包括新建jar file archive 环境变量登资源
-2. 还有脚本开发 包括dws flink python spark hive shell脚本的测试 脚本目录的重命名 移动 删除等操作
+1. 继续对不通的网络进行重新测试
+2. 学习dgc迁移的其他理论知识
 周四:
 1. 1. 进行数据治理的验收测试 主要做的是数据架构验收用例: 比如添加审核人 创建流程设计 导入 导出 删除 创建主题设计 还有概念模型的创建
 2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
@@ -1230,37 +1230,105 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1287,93 +1355,25 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2124,7 +2124,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2148,7 +2148,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2172,7 +2172,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2229,154 +2229,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2385,17 +2385,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2413,15 +2413,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2431,65 +2431,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2499,23 +2516,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/17 周四 17:47:11.68
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B4155A-E223-4220-BB6B-DEDF83FCB6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{064213B5-109D-41E4-BA2F-CF1DE7A30A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,20 +464,20 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>工作&amp;学习日报-9月17日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>重点工作: 
-1. 继续进行dgc迁移工作
+1. 从OBS下载数据开发的内容 然后导入到CDM里面
+2. 继续对不通的网络进行重新测试
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>工作&amp;学习日报-9月16日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>重点工作: 
-1. 继续对不通的网络进行重新测试
-2. 学习dgc迁移的其他理论知识
+1. 继续进行dgc迁移工作和网络测试
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -493,8 +493,7 @@
 1. 继续对不通的网络进行重新测试
 2. 学习dgc迁移的其他理论知识
 周四:
-1. 1. 进行数据治理的验收测试 主要做的是数据架构验收用例: 比如添加审核人 创建流程设计 导入 导出 删除 创建主题设计 还有概念模型的创建
-2. 进行了码表的创建 发布 导出 等工作 以及数仓分层 业务指标的创建 和创建时间限定
+1. 从OBS下载数据开发的内容 然后导入到CDM里面
 周五:
 1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -1230,6 +1229,93 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1283,97 +1369,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2124,7 +2123,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2148,7 +2147,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2172,7 +2171,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2229,154 +2228,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="47"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="47"/>
+      <c r="F2" s="19"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="58"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="21"/>
+      <c r="H3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="41"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2385,17 +2384,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="43"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="34"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2413,15 +2412,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="53"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2431,82 +2430,65 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="28"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="35"/>
+      <c r="J13" s="61"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="22"/>
+      <c r="J14" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2516,6 +2498,23 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/18 周五 17:43:07.74
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{064213B5-109D-41E4-BA2F-CF1DE7A30A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F9A475-D300-4161-8C90-7B39E57E6BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -469,15 +469,15 @@
   </si>
   <si>
     <t>重点工作: 
-1. 从OBS下载数据开发的内容 然后导入到CDM里面
-2. 继续对不通的网络进行重新测试
+1. 登录到大数据集群的后台 查看本地端和北京端的数据量大小 并进行统计增量
+2. 查看数据迁移的日志 统计迁移耗时 根据库的大小 计算速率
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>重点工作: 
-1. 继续进行dgc迁移工作和网络测试
+1. 继续进行dgc迁移工作和MRS增量的迁移工作
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
@@ -495,7 +495,8 @@
 周四:
 1. 从OBS下载数据开发的内容 然后导入到CDM里面
 周五:
-1. 进行了DGC数据服务里的default空间的api发布 和授权操作 以及源端和CDM集群的网络连通行测试</t>
+1. 登录到大数据集群的后台 查看本地端和北京端的数据量大小 并进行统计增量
+2. 查看数据迁移的日志 统计迁移耗时 根据库的大小 计算速率</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
 </sst>
@@ -1229,37 +1230,105 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1286,93 +1355,25 @@
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="165" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="32" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2228,154 +2229,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.75">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="47"/>
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="20"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="58"/>
       <c r="K2" s="9"/>
     </row>
     <row r="3" spans="1:11" ht="15.75">
       <c r="A3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="18" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:11" ht="20.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:11" ht="353" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
     </row>
     <row r="8" spans="1:11" ht="32" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="20.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
     </row>
     <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="2" t="s">
@@ -2384,17 +2385,17 @@
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="40"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="42"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
@@ -2412,15 +2413,15 @@
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="52"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="53"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2430,65 +2431,82 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" customHeight="1">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="56"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:11" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="41" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="60"/>
-      <c r="G13" s="42"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="41" t="s">
+      <c r="I13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:11" ht="14" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="50"/>
+      <c r="J14" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="I14:J14"/>
@@ -2498,23 +2516,6 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:J3"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
更新日报: 2026/09/21 周一 23:22:56.74
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\软通文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F9A475-D300-4161-8C90-7B39E57E6BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC1DF769-0AE4-45F4-BB07-ACF7D84556D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -460,32 +460,32 @@
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
-    <t>2026年9月14日-2026年9月18日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
-    <t>工作&amp;学习日报-9月17日</t>
-    <phoneticPr fontId="30" type="noConversion"/>
-  </si>
-  <si>
     <t>重点工作: 
-1. 登录到大数据集群的后台 查看本地端和北京端的数据量大小 并进行统计增量
-2. 查看数据迁移的日志 统计迁移耗时 根据库的大小 计算速率
+1. 进行MRS的增量迁移和DGC的迁移
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
+    <t>2026年9月20日-2026年9月24日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
+    <t>工作&amp;学习日报-9月21日</t>
+    <phoneticPr fontId="30" type="noConversion"/>
+  </si>
+  <si>
     <t>重点工作: 
-1. 继续进行dgc迁移工作和MRS增量的迁移工作
+1. 进行default工作空间的作业调度的启动和检查操作
+2. 对北京端和目的端的MRS增量数据的统计 并标明哪些增长较快 
 重大风险: 无 
 周边求助: 无</t>
     <phoneticPr fontId="30" type="noConversion"/>
   </si>
   <si>
     <t>周一:
-1. 进行了源端和CDM集群的网络连通行测试
-2. 进行了数据库到源端的连通性 并做了连接 包括oracle postgresql和DM数据库的连接
+1. 进行default工作空间的作业调度的启动和检查操作
+2. 对北京端和目的端的MRS增量数据的统计 并标明哪些增长较快
 周二:
 1. 进行了源端到cdm集群端的网络和端口测试
 2. 从运营面进入数据治理中心  选择工作空间 然后进入数据集成 把dgc里的作业导入到cdm中
@@ -2124,7 +2124,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1">
       <c r="A1" s="65" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B1" s="65"/>
       <c r="C1" s="65"/>
@@ -2148,7 +2148,7 @@
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1">
       <c r="A3" s="68" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="69"/>
@@ -2172,7 +2172,7 @@
     </row>
     <row r="5" spans="1:8" ht="90" customHeight="1">
       <c r="A5" s="71" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B5" s="72"/>
       <c r="C5" s="72"/>
@@ -2261,7 +2261,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="47" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I2" s="47"/>
       <c r="J2" s="58"/>

</xml_diff>